<commit_message>
Add designated authority form checklist item to sabikan pre-employment steps.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/public/downloads/sabikan-checklist.xlsx
+++ b/docs/public/downloads/sabikan-checklist.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="41">
   <si>
     <t>サビ管確認チェックリスト</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t>勤務開始日を確定した</t>
+  </si>
+  <si>
+    <t>各指定権者のフォーマットを渡して記入してもらう</t>
   </si>
   <si>
     <t>指定申請用職員情報を上位店に共有した</t>
@@ -599,7 +602,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -952,21 +955,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+    <row r="39" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-    </row>
-    <row r="41" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="8" t="s">
+      <c r="B39" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C41" s="9"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
     </row>
     <row r="42" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
@@ -985,6 +990,15 @@
         <v>2</v>
       </c>
       <c r="C43" s="9"/>
+    </row>
+    <row r="44" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C44" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -998,10 +1012,10 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="A41:C41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>